<commit_message>
CASE_HEI: GOM-A per spec verbatim + rows 08-07/08-08
GOM-A A1-A5 + GOM-B B1-B4 viết lại per gom_detect_spec v1.4 §1:
- A2: avg5(gLSR)<=1.1 (LEVEL check, không phải slope) — SỬA từ slope<1.0
- A3: glsr_slope_5d<=1.15 (ngưỡng 1.15, không phải 1.0) — SỬA từ pos_r>1.5
- A5: oi_cycle_pos<=0.5 (rolling 30d OI) — MỚI (col 43)
- B1-B4: div_avg3 streak, pin_streak, absorption, NOT funding_neg_div — toàn bộ SỬA
GOM-A fires: 9 ngày (20-24/07, 30-31/07, 01/08, 03/08); GOM-B: 0
07/08 row: partial (fn=3, low_conf=True); 08/08: excluded (chưa đóng 08:35 UTC)
EVENTS row 13: spec-drift line 244 phát hiện 08/08, vá 09/08

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_HEI.xlsx
+++ b/docs/case_files/CASE_HEI.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,9 @@
     <font>
       <b val="1"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="24">
@@ -209,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -291,6 +294,7 @@
     <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1034,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP543"/>
+  <dimension ref="A1:AQ543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="12" min="1" max="1"/>
@@ -1079,6 +1083,7 @@
     <col width="12" customWidth="1" style="12" min="40" max="40"/>
     <col width="12" customWidth="1" style="12" min="41" max="41"/>
     <col width="12" customWidth="1" style="12" min="42" max="42"/>
+    <col width="12" customWidth="1" style="12" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="12">
@@ -1114,12 +1119,17 @@
       </c>
       <c r="AL1" s="31" t="inlineStr">
         <is>
-          <t>GOM SCREEN (gom_detect_spec v1.1 CHUA KY)</t>
+          <t>GOM SCREEN (gom_detect_spec v1.4 ky 08/08)</t>
         </is>
       </c>
       <c r="AO1" s="32" t="inlineStr">
         <is>
           <t>NGUON</t>
+        </is>
+      </c>
+      <c r="AQ1" s="26" t="inlineStr">
+        <is>
+          <t>DERIV-OI (oi_cycle_pos 30d rolling)</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1331,7 @@
       </c>
       <c r="AN2" s="20" t="inlineStr">
         <is>
-          <t>gom_note (CHUA KY)</t>
+          <t>gom_note (spec v1.4 ky 08/08)</t>
         </is>
       </c>
       <c r="AO2" s="20" t="inlineStr">
@@ -1332,6 +1342,11 @@
       <c r="AP2" s="20" t="inlineStr">
         <is>
           <t>data_source_lsr</t>
+        </is>
+      </c>
+      <c r="AQ2" s="20" t="inlineStr">
+        <is>
+          <t>oi_cycle_pos (rolling 30d OI window)</t>
         </is>
       </c>
     </row>
@@ -1434,6 +1449,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ3" s="21" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
@@ -1536,6 +1552,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ4" s="21" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
@@ -1638,6 +1655,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ5" s="21" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
@@ -1740,6 +1758,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ6" s="21" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
@@ -1842,6 +1861,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ7" s="21" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
@@ -1944,6 +1964,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ8" s="21" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
@@ -2046,6 +2067,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ9" s="21" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
@@ -2148,6 +2170,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ10" s="21" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
@@ -2250,6 +2273,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ11" s="21" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
@@ -2352,6 +2376,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ12" s="21" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
@@ -2454,6 +2479,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ13" s="21" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
@@ -2556,6 +2582,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ14" s="21" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
@@ -2658,6 +2685,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ15" s="21" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
@@ -2760,6 +2788,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ16" s="21" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="21" t="inlineStr">
@@ -2864,6 +2893,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ17" s="21" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="21" t="inlineStr">
@@ -2968,6 +2998,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ18" s="21" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="21" t="inlineStr">
@@ -3072,6 +3103,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ19" s="21" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
@@ -3176,6 +3208,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ20" s="21" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
@@ -3280,6 +3313,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ21" s="21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
@@ -3384,6 +3418,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ22" s="21" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
@@ -3488,6 +3523,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ23" s="21" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
@@ -3592,6 +3628,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ24" s="21" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="21" t="inlineStr">
@@ -3696,6 +3733,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ25" s="21" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
@@ -3800,6 +3838,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ26" s="21" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
@@ -3904,6 +3943,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ27" s="21" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
@@ -4008,6 +4048,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ28" s="21" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
@@ -4112,6 +4153,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ29" s="21" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
@@ -4216,6 +4258,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ30" s="21" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
@@ -4320,6 +4363,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ31" s="21" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
@@ -4424,6 +4468,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ32" s="21" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
@@ -4528,6 +4573,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ33" s="21" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
@@ -4632,6 +4678,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ34" s="21" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
@@ -4736,6 +4783,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ35" s="21" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
@@ -4840,6 +4888,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ36" s="21" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
@@ -4944,6 +4993,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ37" s="21" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
@@ -5048,6 +5098,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ38" s="21" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="21" t="inlineStr">
@@ -5152,6 +5203,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ39" s="21" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
@@ -5256,6 +5308,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ40" s="21" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
@@ -5360,6 +5413,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ41" s="21" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
@@ -5464,6 +5518,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ42" s="21" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
@@ -5568,6 +5623,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ43" s="21" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
@@ -5672,6 +5728,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ44" s="21" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
@@ -5776,6 +5833,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ45" s="21" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
@@ -5880,6 +5938,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ46" s="21" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
@@ -5984,6 +6043,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ47" s="21" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
@@ -6088,6 +6148,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ48" s="21" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="21" t="inlineStr">
@@ -6192,6 +6253,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ49" s="21" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
@@ -6296,6 +6358,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ50" s="21" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
@@ -6400,6 +6463,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ51" s="21" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
@@ -6504,6 +6568,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ52" s="21" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="21" t="inlineStr">
@@ -6608,6 +6673,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ53" s="21" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
@@ -6712,6 +6778,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ54" s="21" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
@@ -6816,6 +6883,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ55" s="21" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="21" t="inlineStr">
@@ -6920,6 +6988,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ56" s="21" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="21" t="inlineStr">
@@ -7024,6 +7093,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ57" s="21" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="21" t="inlineStr">
@@ -7128,6 +7198,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ58" s="21" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="21" t="inlineStr">
@@ -7232,6 +7303,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ59" s="21" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="21" t="inlineStr">
@@ -7336,6 +7408,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ60" s="21" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="21" t="inlineStr">
@@ -7440,6 +7513,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ61" s="21" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="21" t="inlineStr">
@@ -7544,6 +7618,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ62" s="21" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
@@ -7648,6 +7723,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ63" s="21" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
@@ -7752,6 +7828,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ64" s="21" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="21" t="inlineStr">
@@ -7856,6 +7933,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ65" s="21" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="21" t="inlineStr">
@@ -7960,6 +8038,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ66" s="21" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="21" t="inlineStr">
@@ -8064,6 +8143,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ67" s="21" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="21" t="inlineStr">
@@ -8168,6 +8248,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ68" s="21" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="21" t="inlineStr">
@@ -8272,6 +8353,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ69" s="21" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="21" t="inlineStr">
@@ -8376,6 +8458,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ70" s="21" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="21" t="inlineStr">
@@ -8480,6 +8563,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ71" s="21" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="21" t="inlineStr">
@@ -8584,6 +8668,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ72" s="21" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="21" t="inlineStr">
@@ -8688,6 +8773,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ73" s="21" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="21" t="inlineStr">
@@ -8792,6 +8878,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ74" s="21" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="21" t="inlineStr">
@@ -8896,6 +8983,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ75" s="21" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="21" t="inlineStr">
@@ -9000,6 +9088,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ76" s="21" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="21" t="inlineStr">
@@ -9104,6 +9193,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ77" s="21" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="21" t="inlineStr">
@@ -9208,6 +9298,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ78" s="21" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="21" t="inlineStr">
@@ -9312,6 +9403,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ79" s="21" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="21" t="inlineStr">
@@ -9416,6 +9508,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ80" s="21" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="21" t="inlineStr">
@@ -9520,6 +9613,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ81" s="21" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="21" t="inlineStr">
@@ -9624,6 +9718,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ82" s="21" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="21" t="inlineStr">
@@ -9728,6 +9823,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ83" s="21" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="21" t="inlineStr">
@@ -9832,6 +9928,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ84" s="21" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="21" t="inlineStr">
@@ -9936,6 +10033,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ85" s="21" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="21" t="inlineStr">
@@ -10040,6 +10138,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ86" s="21" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="21" t="inlineStr">
@@ -10144,6 +10243,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ87" s="21" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="21" t="inlineStr">
@@ -10248,6 +10348,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ88" s="21" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="21" t="inlineStr">
@@ -10352,6 +10453,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ89" s="21" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="21" t="inlineStr">
@@ -10456,6 +10558,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ90" s="21" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="21" t="inlineStr">
@@ -10560,6 +10663,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ91" s="21" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="21" t="inlineStr">
@@ -10664,6 +10768,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ92" s="21" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="21" t="inlineStr">
@@ -10768,6 +10873,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ93" s="21" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="21" t="inlineStr">
@@ -10872,6 +10978,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ94" s="21" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="21" t="inlineStr">
@@ -10976,6 +11083,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ95" s="21" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="21" t="inlineStr">
@@ -11080,6 +11188,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ96" s="21" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="21" t="inlineStr">
@@ -11184,6 +11293,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ97" s="21" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
@@ -11288,6 +11398,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ98" s="21" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="21" t="inlineStr">
@@ -11392,6 +11503,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ99" s="21" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="21" t="inlineStr">
@@ -11496,6 +11608,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ100" s="21" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="21" t="inlineStr">
@@ -11600,6 +11713,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ101" s="21" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="21" t="inlineStr">
@@ -11704,6 +11818,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ102" s="21" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="21" t="inlineStr">
@@ -11808,6 +11923,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ103" s="21" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="21" t="inlineStr">
@@ -11912,6 +12028,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ104" s="21" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="21" t="inlineStr">
@@ -12016,6 +12133,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ105" s="21" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="21" t="inlineStr">
@@ -12120,6 +12238,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ106" s="21" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="21" t="inlineStr">
@@ -12224,6 +12343,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ107" s="21" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="21" t="inlineStr">
@@ -12328,6 +12448,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ108" s="21" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="21" t="inlineStr">
@@ -12432,6 +12553,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ109" s="21" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="21" t="inlineStr">
@@ -12536,6 +12658,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ110" s="21" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="21" t="inlineStr">
@@ -12640,6 +12763,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ111" s="21" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="21" t="inlineStr">
@@ -12744,6 +12868,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ112" s="21" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="21" t="inlineStr">
@@ -12848,6 +12973,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ113" s="21" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="21" t="inlineStr">
@@ -12952,6 +13078,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ114" s="21" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="21" t="inlineStr">
@@ -13056,6 +13183,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ115" s="21" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="21" t="inlineStr">
@@ -13160,6 +13288,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ116" s="21" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="21" t="inlineStr">
@@ -13264,6 +13393,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ117" s="21" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="21" t="inlineStr">
@@ -13368,6 +13498,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ118" s="21" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="21" t="inlineStr">
@@ -13472,6 +13603,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ119" s="21" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="21" t="inlineStr">
@@ -13576,6 +13708,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ120" s="21" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="21" t="inlineStr">
@@ -13680,6 +13813,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ121" s="21" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="21" t="inlineStr">
@@ -13784,6 +13918,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ122" s="21" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="21" t="inlineStr">
@@ -13888,6 +14023,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ123" s="21" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="21" t="inlineStr">
@@ -13992,6 +14128,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ124" s="21" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="21" t="inlineStr">
@@ -14096,6 +14233,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ125" s="21" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="21" t="inlineStr">
@@ -14200,6 +14338,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ126" s="21" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="21" t="inlineStr">
@@ -14304,6 +14443,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ127" s="21" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="21" t="inlineStr">
@@ -14408,6 +14548,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ128" s="21" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="21" t="inlineStr">
@@ -14512,6 +14653,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ129" s="21" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="21" t="inlineStr">
@@ -14616,6 +14758,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ130" s="21" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="21" t="inlineStr">
@@ -14720,6 +14863,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ131" s="21" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="21" t="inlineStr">
@@ -14824,6 +14968,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ132" s="21" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="21" t="inlineStr">
@@ -14928,6 +15073,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ133" s="21" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="21" t="inlineStr">
@@ -15032,6 +15178,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ134" s="21" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="21" t="inlineStr">
@@ -15136,6 +15283,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ135" s="21" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="21" t="inlineStr">
@@ -15240,6 +15388,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ136" s="21" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="21" t="inlineStr">
@@ -15344,6 +15493,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ137" s="21" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="21" t="inlineStr">
@@ -15448,6 +15598,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ138" s="21" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="21" t="inlineStr">
@@ -15552,6 +15703,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ139" s="21" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="21" t="inlineStr">
@@ -15656,6 +15808,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ140" s="21" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="21" t="inlineStr">
@@ -15760,6 +15913,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ141" s="21" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
@@ -15864,6 +16018,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ142" s="21" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="21" t="inlineStr">
@@ -15968,6 +16123,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ143" s="21" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="21" t="inlineStr">
@@ -16072,6 +16228,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ144" s="21" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="21" t="inlineStr">
@@ -16176,6 +16333,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ145" s="21" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="21" t="inlineStr">
@@ -16280,6 +16438,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ146" s="21" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="21" t="inlineStr">
@@ -16384,6 +16543,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ147" s="21" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="21" t="inlineStr">
@@ -16488,6 +16648,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ148" s="21" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="21" t="inlineStr">
@@ -16592,6 +16753,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ149" s="21" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="21" t="inlineStr">
@@ -16696,6 +16858,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ150" s="21" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="21" t="inlineStr">
@@ -16800,6 +16963,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ151" s="21" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="21" t="inlineStr">
@@ -16904,6 +17068,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ152" s="21" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="21" t="inlineStr">
@@ -17008,6 +17173,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ153" s="21" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="21" t="inlineStr">
@@ -17112,6 +17278,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ154" s="21" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="21" t="inlineStr">
@@ -17216,6 +17383,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ155" s="21" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="21" t="inlineStr">
@@ -17320,6 +17488,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ156" s="21" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="21" t="inlineStr">
@@ -17424,6 +17593,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ157" s="21" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="21" t="inlineStr">
@@ -17528,6 +17698,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ158" s="21" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="21" t="inlineStr">
@@ -17632,6 +17803,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ159" s="21" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="21" t="inlineStr">
@@ -17736,6 +17908,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ160" s="21" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="21" t="inlineStr">
@@ -17840,6 +18013,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ161" s="21" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="21" t="inlineStr">
@@ -17944,6 +18118,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ162" s="21" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="21" t="inlineStr">
@@ -18048,6 +18223,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ163" s="21" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="21" t="inlineStr">
@@ -18152,6 +18328,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ164" s="21" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="21" t="inlineStr">
@@ -18256,6 +18433,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ165" s="21" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="21" t="inlineStr">
@@ -18360,6 +18538,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ166" s="21" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="21" t="inlineStr">
@@ -18464,6 +18643,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ167" s="21" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="21" t="inlineStr">
@@ -18568,6 +18748,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ168" s="21" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="21" t="inlineStr">
@@ -18672,6 +18853,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ169" s="21" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="21" t="inlineStr">
@@ -18776,6 +18958,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ170" s="21" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="21" t="inlineStr">
@@ -18880,6 +19063,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ171" s="21" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="21" t="inlineStr">
@@ -18984,6 +19168,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ172" s="21" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="21" t="inlineStr">
@@ -19088,6 +19273,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ173" s="21" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="21" t="inlineStr">
@@ -19192,6 +19378,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ174" s="21" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="21" t="inlineStr">
@@ -19296,6 +19483,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ175" s="21" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="21" t="inlineStr">
@@ -19400,6 +19588,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ176" s="21" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="21" t="inlineStr">
@@ -19504,6 +19693,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ177" s="21" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="21" t="inlineStr">
@@ -19608,6 +19798,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ178" s="21" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="21" t="inlineStr">
@@ -19712,6 +19903,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ179" s="21" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="21" t="inlineStr">
@@ -19816,6 +20008,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ180" s="21" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="21" t="inlineStr">
@@ -19920,6 +20113,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ181" s="21" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="21" t="inlineStr">
@@ -20024,6 +20218,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ182" s="21" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="21" t="inlineStr">
@@ -20128,6 +20323,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ183" s="21" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="21" t="inlineStr">
@@ -20232,6 +20428,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ184" s="21" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="21" t="inlineStr">
@@ -20336,6 +20533,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ185" s="21" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="21" t="inlineStr">
@@ -20440,6 +20638,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ186" s="21" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="21" t="inlineStr">
@@ -20544,6 +20743,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ187" s="21" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="21" t="inlineStr">
@@ -20648,6 +20848,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ188" s="21" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="21" t="inlineStr">
@@ -20752,6 +20953,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ189" s="21" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="21" t="inlineStr">
@@ -20856,6 +21058,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ190" s="21" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="21" t="inlineStr">
@@ -20960,6 +21163,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ191" s="21" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="21" t="inlineStr">
@@ -21064,6 +21268,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ192" s="21" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="21" t="inlineStr">
@@ -21168,6 +21373,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ193" s="21" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="21" t="inlineStr">
@@ -21272,6 +21478,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ194" s="21" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="21" t="inlineStr">
@@ -21376,6 +21583,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ195" s="21" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="21" t="inlineStr">
@@ -21480,6 +21688,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ196" s="21" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="21" t="inlineStr">
@@ -21584,6 +21793,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ197" s="21" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="21" t="inlineStr">
@@ -21688,6 +21898,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ198" s="21" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="21" t="inlineStr">
@@ -21792,6 +22003,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ199" s="21" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="21" t="inlineStr">
@@ -21896,6 +22108,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ200" s="21" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="21" t="inlineStr">
@@ -22000,6 +22213,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ201" s="21" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="21" t="inlineStr">
@@ -22104,6 +22318,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ202" s="21" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="21" t="inlineStr">
@@ -22208,6 +22423,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ203" s="21" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="21" t="inlineStr">
@@ -22312,6 +22528,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ204" s="21" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="21" t="inlineStr">
@@ -22416,6 +22633,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ205" s="21" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="21" t="inlineStr">
@@ -22520,6 +22738,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ206" s="21" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="21" t="inlineStr">
@@ -22624,6 +22843,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ207" s="21" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="21" t="inlineStr">
@@ -22728,6 +22948,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ208" s="21" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="21" t="inlineStr">
@@ -22832,6 +23053,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ209" s="21" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="21" t="inlineStr">
@@ -22936,6 +23158,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ210" s="21" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="21" t="inlineStr">
@@ -23040,6 +23263,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ211" s="21" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="21" t="inlineStr">
@@ -23144,6 +23368,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ212" s="21" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="21" t="inlineStr">
@@ -23248,6 +23473,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ213" s="21" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="21" t="inlineStr">
@@ -23352,6 +23578,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ214" s="21" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="21" t="inlineStr">
@@ -23456,6 +23683,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ215" s="21" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="21" t="inlineStr">
@@ -23560,6 +23788,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ216" s="21" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="21" t="inlineStr">
@@ -23664,6 +23893,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ217" s="21" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="21" t="inlineStr">
@@ -23768,6 +23998,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ218" s="21" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="21" t="inlineStr">
@@ -23872,6 +24103,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ219" s="21" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="21" t="inlineStr">
@@ -23976,6 +24208,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ220" s="21" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="21" t="inlineStr">
@@ -24080,6 +24313,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ221" s="21" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="21" t="inlineStr">
@@ -24184,6 +24418,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ222" s="21" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="21" t="inlineStr">
@@ -24288,6 +24523,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ223" s="21" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="21" t="inlineStr">
@@ -24392,6 +24628,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ224" s="21" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="21" t="inlineStr">
@@ -24496,6 +24733,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ225" s="21" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="21" t="inlineStr">
@@ -24600,6 +24838,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ226" s="21" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="21" t="inlineStr">
@@ -24704,6 +24943,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ227" s="21" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="21" t="inlineStr">
@@ -24808,6 +25048,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ228" s="21" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="21" t="inlineStr">
@@ -24912,6 +25153,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ229" s="21" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="21" t="inlineStr">
@@ -25016,6 +25258,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ230" s="21" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="21" t="inlineStr">
@@ -25120,6 +25363,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ231" s="21" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="21" t="inlineStr">
@@ -25224,6 +25468,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ232" s="21" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="21" t="inlineStr">
@@ -25328,6 +25573,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ233" s="21" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="21" t="inlineStr">
@@ -25432,6 +25678,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ234" s="21" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="21" t="inlineStr">
@@ -25536,6 +25783,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ235" s="21" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="21" t="inlineStr">
@@ -25640,6 +25888,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ236" s="21" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="21" t="inlineStr">
@@ -25744,6 +25993,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ237" s="21" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="21" t="inlineStr">
@@ -25848,6 +26098,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ238" s="21" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="21" t="inlineStr">
@@ -25952,6 +26203,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ239" s="21" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="21" t="inlineStr">
@@ -26056,6 +26308,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ240" s="21" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="21" t="inlineStr">
@@ -26160,6 +26413,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ241" s="21" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="21" t="inlineStr">
@@ -26264,6 +26518,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ242" s="21" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="21" t="inlineStr">
@@ -26368,6 +26623,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ243" s="21" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="21" t="inlineStr">
@@ -26472,6 +26728,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ244" s="21" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="21" t="inlineStr">
@@ -26576,6 +26833,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ245" s="21" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="21" t="inlineStr">
@@ -26680,6 +26938,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ246" s="21" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="21" t="inlineStr">
@@ -26784,6 +27043,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ247" s="21" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="21" t="inlineStr">
@@ -26888,6 +27148,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ248" s="21" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="21" t="inlineStr">
@@ -26992,6 +27253,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ249" s="21" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="21" t="inlineStr">
@@ -27096,6 +27358,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ250" s="21" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="21" t="inlineStr">
@@ -27200,6 +27463,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ251" s="21" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="21" t="inlineStr">
@@ -27304,6 +27568,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ252" s="21" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="21" t="inlineStr">
@@ -27408,6 +27673,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ253" s="21" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="21" t="inlineStr">
@@ -27512,6 +27778,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ254" s="21" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="21" t="inlineStr">
@@ -27616,6 +27883,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ255" s="21" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="21" t="inlineStr">
@@ -27720,6 +27988,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ256" s="21" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="21" t="inlineStr">
@@ -27824,6 +28093,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ257" s="21" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="21" t="inlineStr">
@@ -27928,6 +28198,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ258" s="21" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="21" t="inlineStr">
@@ -28032,6 +28303,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ259" s="21" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="21" t="inlineStr">
@@ -28136,6 +28408,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ260" s="21" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="21" t="inlineStr">
@@ -28240,6 +28513,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ261" s="21" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="21" t="inlineStr">
@@ -28344,6 +28618,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ262" s="21" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="21" t="inlineStr">
@@ -28448,6 +28723,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ263" s="21" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="21" t="inlineStr">
@@ -28552,6 +28828,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ264" s="21" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="21" t="inlineStr">
@@ -28656,6 +28933,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ265" s="21" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="21" t="inlineStr">
@@ -28760,6 +29038,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ266" s="21" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="21" t="inlineStr">
@@ -28864,6 +29143,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ267" s="21" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="21" t="inlineStr">
@@ -28968,6 +29248,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ268" s="21" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="21" t="inlineStr">
@@ -29072,6 +29353,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ269" s="21" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="21" t="inlineStr">
@@ -29176,6 +29458,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ270" s="21" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="21" t="inlineStr">
@@ -29280,6 +29563,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ271" s="21" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="21" t="inlineStr">
@@ -29384,6 +29668,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ272" s="21" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="21" t="inlineStr">
@@ -29488,6 +29773,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ273" s="21" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="21" t="inlineStr">
@@ -29592,6 +29878,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ274" s="21" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="21" t="inlineStr">
@@ -29696,6 +29983,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ275" s="21" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="21" t="inlineStr">
@@ -29800,6 +30088,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ276" s="21" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="21" t="inlineStr">
@@ -29904,6 +30193,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ277" s="21" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="21" t="inlineStr">
@@ -30008,6 +30298,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ278" s="21" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="21" t="inlineStr">
@@ -30112,6 +30403,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ279" s="21" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="21" t="inlineStr">
@@ -30216,6 +30508,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ280" s="21" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="21" t="inlineStr">
@@ -30320,6 +30613,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ281" s="21" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="21" t="inlineStr">
@@ -30424,6 +30718,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ282" s="21" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="21" t="inlineStr">
@@ -30528,6 +30823,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ283" s="21" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="21" t="inlineStr">
@@ -30632,6 +30928,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ284" s="21" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="21" t="inlineStr">
@@ -30736,6 +31033,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ285" s="21" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" s="21" t="inlineStr">
@@ -30840,6 +31138,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ286" s="21" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="21" t="inlineStr">
@@ -30944,6 +31243,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ287" s="21" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="21" t="inlineStr">
@@ -31048,6 +31348,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ288" s="21" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" s="21" t="inlineStr">
@@ -31152,6 +31453,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ289" s="21" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" s="21" t="inlineStr">
@@ -31256,6 +31558,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ290" s="21" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="21" t="inlineStr">
@@ -31360,6 +31663,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ291" s="21" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" s="21" t="inlineStr">
@@ -31464,6 +31768,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ292" s="21" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" s="21" t="inlineStr">
@@ -31568,6 +31873,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ293" s="21" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" s="21" t="inlineStr">
@@ -31672,6 +31978,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ294" s="21" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="21" t="inlineStr">
@@ -31776,6 +32083,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ295" s="21" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="21" t="inlineStr">
@@ -31880,6 +32188,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ296" s="21" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="21" t="inlineStr">
@@ -31984,6 +32293,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ297" s="21" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="21" t="inlineStr">
@@ -32088,6 +32398,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ298" s="21" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="21" t="inlineStr">
@@ -32192,6 +32503,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ299" s="21" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="21" t="inlineStr">
@@ -32296,6 +32608,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ300" s="21" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" s="21" t="inlineStr">
@@ -32400,6 +32713,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ301" s="21" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" s="21" t="inlineStr">
@@ -32504,6 +32818,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ302" s="21" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" s="21" t="inlineStr">
@@ -32608,6 +32923,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ303" s="21" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" s="21" t="inlineStr">
@@ -32712,6 +33028,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ304" s="21" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" s="21" t="inlineStr">
@@ -32816,6 +33133,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ305" s="21" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" s="21" t="inlineStr">
@@ -32920,6 +33238,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ306" s="21" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="21" t="inlineStr">
@@ -33024,6 +33343,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ307" s="21" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="21" t="inlineStr">
@@ -33128,6 +33448,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ308" s="21" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" s="21" t="inlineStr">
@@ -33232,6 +33553,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ309" s="21" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" s="21" t="inlineStr">
@@ -33336,6 +33658,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ310" s="21" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" s="21" t="inlineStr">
@@ -33440,6 +33763,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ311" s="21" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" s="21" t="inlineStr">
@@ -33544,6 +33868,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ312" s="21" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" s="21" t="inlineStr">
@@ -33648,6 +33973,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ313" s="21" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="21" t="inlineStr">
@@ -33752,6 +34078,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ314" s="21" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="21" t="inlineStr">
@@ -33856,6 +34183,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ315" s="21" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="21" t="inlineStr">
@@ -33960,6 +34288,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ316" s="21" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" s="21" t="inlineStr">
@@ -34064,6 +34393,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ317" s="21" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" s="21" t="inlineStr">
@@ -34168,6 +34498,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ318" s="21" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" s="21" t="inlineStr">
@@ -34272,6 +34603,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ319" s="21" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" s="21" t="inlineStr">
@@ -34376,6 +34708,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ320" s="21" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" s="21" t="inlineStr">
@@ -34480,6 +34813,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ321" s="21" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" s="21" t="inlineStr">
@@ -34584,6 +34918,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ322" s="21" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="21" t="inlineStr">
@@ -34688,6 +35023,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ323" s="21" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" s="21" t="inlineStr">
@@ -34792,6 +35128,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ324" s="21" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" s="21" t="inlineStr">
@@ -34896,6 +35233,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ325" s="21" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" s="21" t="inlineStr">
@@ -35000,6 +35338,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ326" s="21" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" s="21" t="inlineStr">
@@ -35104,6 +35443,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ327" s="21" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" s="21" t="inlineStr">
@@ -35208,6 +35548,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ328" s="21" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" s="21" t="inlineStr">
@@ -35312,6 +35653,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ329" s="21" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" s="21" t="inlineStr">
@@ -35416,6 +35758,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ330" s="21" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" s="21" t="inlineStr">
@@ -35520,6 +35863,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ331" s="21" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" s="21" t="inlineStr">
@@ -35624,6 +35968,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ332" s="21" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" s="21" t="inlineStr">
@@ -35728,6 +36073,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ333" s="21" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" s="21" t="inlineStr">
@@ -35832,6 +36178,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ334" s="21" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" s="21" t="inlineStr">
@@ -35936,6 +36283,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ335" s="21" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" s="21" t="inlineStr">
@@ -36040,6 +36388,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ336" s="21" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" s="21" t="inlineStr">
@@ -36144,6 +36493,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ337" s="21" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" s="21" t="inlineStr">
@@ -36248,6 +36598,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ338" s="21" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" s="21" t="inlineStr">
@@ -36352,6 +36703,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ339" s="21" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" s="21" t="inlineStr">
@@ -36456,6 +36808,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ340" s="21" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" s="21" t="inlineStr">
@@ -36560,6 +36913,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ341" s="21" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" s="21" t="inlineStr">
@@ -36664,6 +37018,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ342" s="21" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="21" t="inlineStr">
@@ -36768,6 +37123,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ343" s="21" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" s="21" t="inlineStr">
@@ -36872,6 +37228,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ344" s="21" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" s="21" t="inlineStr">
@@ -36976,6 +37333,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ345" s="21" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" s="21" t="inlineStr">
@@ -37080,6 +37438,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ346" s="21" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" s="21" t="inlineStr">
@@ -37184,6 +37543,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ347" s="21" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" s="21" t="inlineStr">
@@ -37288,6 +37648,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ348" s="21" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" s="21" t="inlineStr">
@@ -37392,6 +37753,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ349" s="21" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" s="21" t="inlineStr">
@@ -37496,6 +37858,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ350" s="21" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" s="21" t="inlineStr">
@@ -37600,6 +37963,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ351" s="21" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" s="21" t="inlineStr">
@@ -37704,6 +38068,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ352" s="21" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" s="21" t="inlineStr">
@@ -37808,6 +38173,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ353" s="21" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" s="21" t="inlineStr">
@@ -37912,6 +38278,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ354" s="21" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" s="21" t="inlineStr">
@@ -38016,6 +38383,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ355" s="21" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" s="21" t="inlineStr">
@@ -38120,6 +38488,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ356" s="21" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" s="21" t="inlineStr">
@@ -38224,6 +38593,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ357" s="21" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" s="21" t="inlineStr">
@@ -38328,6 +38698,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ358" s="21" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" s="21" t="inlineStr">
@@ -38432,6 +38803,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ359" s="21" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" s="21" t="inlineStr">
@@ -38536,6 +38908,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ360" s="21" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" s="21" t="inlineStr">
@@ -38640,6 +39013,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ361" s="21" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="21" t="inlineStr">
@@ -38744,6 +39118,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ362" s="21" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" s="21" t="inlineStr">
@@ -38848,6 +39223,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ363" s="21" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" s="21" t="inlineStr">
@@ -38952,6 +39328,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ364" s="21" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" s="21" t="inlineStr">
@@ -39056,6 +39433,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ365" s="21" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" s="21" t="inlineStr">
@@ -39160,6 +39538,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ366" s="21" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" s="21" t="inlineStr">
@@ -39264,6 +39643,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ367" s="21" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" s="21" t="inlineStr">
@@ -39368,6 +39748,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ368" s="21" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" s="21" t="inlineStr">
@@ -39472,6 +39853,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ369" s="21" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" s="21" t="inlineStr">
@@ -39576,6 +39958,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ370" s="21" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" s="21" t="inlineStr">
@@ -39680,6 +40063,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ371" s="21" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" s="21" t="inlineStr">
@@ -39784,6 +40168,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ372" s="21" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" s="21" t="inlineStr">
@@ -39888,6 +40273,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ373" s="21" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" s="21" t="inlineStr">
@@ -39992,6 +40378,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ374" s="21" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" s="21" t="inlineStr">
@@ -40096,6 +40483,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ375" s="21" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" s="21" t="inlineStr">
@@ -40200,6 +40588,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ376" s="21" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" s="21" t="inlineStr">
@@ -40304,6 +40693,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ377" s="21" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" s="21" t="inlineStr">
@@ -40408,6 +40798,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ378" s="21" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" s="21" t="inlineStr">
@@ -40512,6 +40903,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ379" s="21" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" s="21" t="inlineStr">
@@ -40616,6 +41008,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ380" s="21" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" s="21" t="inlineStr">
@@ -40720,6 +41113,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ381" s="21" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" s="21" t="inlineStr">
@@ -40824,6 +41218,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ382" s="21" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" s="21" t="inlineStr">
@@ -40928,6 +41323,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ383" s="21" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" s="21" t="inlineStr">
@@ -41032,6 +41428,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ384" s="21" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" s="21" t="inlineStr">
@@ -41136,6 +41533,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ385" s="21" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" s="21" t="inlineStr">
@@ -41240,6 +41638,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ386" s="21" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" s="21" t="inlineStr">
@@ -41344,6 +41743,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ387" s="21" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" s="21" t="inlineStr">
@@ -41448,6 +41848,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ388" s="21" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" s="21" t="inlineStr">
@@ -41552,6 +41953,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ389" s="21" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" s="21" t="inlineStr">
@@ -41656,6 +42058,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ390" s="21" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" s="21" t="inlineStr">
@@ -41760,6 +42163,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ391" s="21" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" s="21" t="inlineStr">
@@ -41864,6 +42268,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ392" s="21" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" s="21" t="inlineStr">
@@ -41968,6 +42373,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ393" s="21" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" s="21" t="inlineStr">
@@ -42072,6 +42478,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ394" s="21" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" s="21" t="inlineStr">
@@ -42176,6 +42583,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ395" s="21" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" s="21" t="inlineStr">
@@ -42280,6 +42688,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ396" s="21" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" s="21" t="inlineStr">
@@ -42384,6 +42793,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ397" s="21" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" s="21" t="inlineStr">
@@ -42488,6 +42898,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ398" s="21" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" s="21" t="inlineStr">
@@ -42592,6 +43003,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ399" s="21" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" s="21" t="inlineStr">
@@ -42696,6 +43108,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ400" s="21" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" s="21" t="inlineStr">
@@ -42800,6 +43213,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ401" s="21" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" s="21" t="inlineStr">
@@ -42904,6 +43318,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ402" s="21" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" s="21" t="inlineStr">
@@ -43008,6 +43423,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ403" s="21" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" s="21" t="inlineStr">
@@ -43112,6 +43528,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ404" s="21" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" s="21" t="inlineStr">
@@ -43216,6 +43633,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ405" s="21" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" s="21" t="inlineStr">
@@ -43320,6 +43738,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ406" s="21" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" s="21" t="inlineStr">
@@ -43424,6 +43843,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ407" s="21" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" s="21" t="inlineStr">
@@ -43528,6 +43948,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ408" s="21" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" s="21" t="inlineStr">
@@ -43632,6 +44053,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ409" s="21" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" s="21" t="inlineStr">
@@ -43736,6 +44158,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ410" s="21" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" s="21" t="inlineStr">
@@ -43840,6 +44263,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ411" s="21" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" s="21" t="inlineStr">
@@ -43944,6 +44368,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ412" s="21" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" s="21" t="inlineStr">
@@ -44048,6 +44473,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ413" s="21" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" s="21" t="inlineStr">
@@ -44152,6 +44578,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ414" s="21" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" s="21" t="inlineStr">
@@ -44256,6 +44683,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ415" s="21" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" s="21" t="inlineStr">
@@ -44360,6 +44788,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ416" s="21" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" s="21" t="inlineStr">
@@ -44464,6 +44893,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ417" s="21" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" s="21" t="inlineStr">
@@ -44568,6 +44998,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ418" s="21" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" s="21" t="inlineStr">
@@ -44672,6 +45103,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ419" s="21" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" s="21" t="inlineStr">
@@ -44776,6 +45208,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ420" s="21" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" s="21" t="inlineStr">
@@ -44880,6 +45313,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ421" s="21" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" s="21" t="inlineStr">
@@ -44984,6 +45418,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ422" s="21" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" s="21" t="inlineStr">
@@ -45088,6 +45523,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ423" s="21" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" s="21" t="inlineStr">
@@ -45192,6 +45628,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ424" s="21" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" s="21" t="inlineStr">
@@ -45296,6 +45733,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ425" s="21" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" s="21" t="inlineStr">
@@ -45400,6 +45838,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ426" s="21" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" s="21" t="inlineStr">
@@ -45504,6 +45943,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ427" s="21" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" s="21" t="inlineStr">
@@ -45608,6 +46048,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ428" s="21" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" s="21" t="inlineStr">
@@ -45712,6 +46153,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ429" s="21" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" s="21" t="inlineStr">
@@ -45816,6 +46258,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ430" s="21" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" s="21" t="inlineStr">
@@ -45920,6 +46363,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ431" s="21" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" s="21" t="inlineStr">
@@ -46024,6 +46468,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ432" s="21" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" s="21" t="inlineStr">
@@ -46128,6 +46573,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ433" s="21" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" s="21" t="inlineStr">
@@ -46232,6 +46678,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ434" s="21" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" s="21" t="inlineStr">
@@ -46336,6 +46783,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ435" s="21" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" s="21" t="inlineStr">
@@ -46440,6 +46888,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ436" s="21" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" s="21" t="inlineStr">
@@ -46544,6 +46993,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ437" s="21" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" s="21" t="inlineStr">
@@ -46648,6 +47098,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ438" s="21" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" s="21" t="inlineStr">
@@ -46752,6 +47203,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ439" s="21" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" s="21" t="inlineStr">
@@ -46856,6 +47308,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ440" s="21" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" s="21" t="inlineStr">
@@ -46960,6 +47413,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ441" s="21" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" s="21" t="inlineStr">
@@ -47064,6 +47518,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ442" s="21" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" s="21" t="inlineStr">
@@ -47168,6 +47623,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ443" s="21" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" s="21" t="inlineStr">
@@ -47272,6 +47728,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ444" s="21" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" s="21" t="inlineStr">
@@ -47376,6 +47833,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ445" s="21" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" s="21" t="inlineStr">
@@ -47480,6 +47938,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ446" s="21" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" s="21" t="inlineStr">
@@ -47584,6 +48043,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ447" s="21" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" s="21" t="inlineStr">
@@ -47688,6 +48148,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ448" s="21" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" s="21" t="inlineStr">
@@ -47792,6 +48253,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ449" s="21" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" s="21" t="inlineStr">
@@ -47896,6 +48358,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ450" s="21" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" s="21" t="inlineStr">
@@ -48000,6 +48463,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ451" s="21" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" s="21" t="inlineStr">
@@ -48104,6 +48568,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ452" s="21" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" s="21" t="inlineStr">
@@ -48208,6 +48673,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ453" s="21" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" s="21" t="inlineStr">
@@ -48312,6 +48778,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ454" s="21" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" s="21" t="inlineStr">
@@ -48416,6 +48883,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ455" s="21" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" s="21" t="inlineStr">
@@ -48520,6 +48988,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ456" s="21" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" s="21" t="inlineStr">
@@ -48624,6 +49093,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ457" s="21" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" s="21" t="inlineStr">
@@ -48728,6 +49198,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ458" s="21" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" s="21" t="inlineStr">
@@ -48832,6 +49303,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ459" s="21" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" s="21" t="inlineStr">
@@ -48936,6 +49408,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ460" s="21" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" s="21" t="inlineStr">
@@ -49040,6 +49513,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ461" s="21" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" s="21" t="inlineStr">
@@ -49156,6 +49630,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ462" s="21" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" s="21" t="inlineStr">
@@ -49272,6 +49747,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ463" s="21" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" s="21" t="inlineStr">
@@ -49388,6 +49864,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ464" s="21" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" s="21" t="inlineStr">
@@ -49504,6 +49981,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ465" s="21" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" s="21" t="inlineStr">
@@ -49620,6 +50098,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ466" s="21" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" s="21" t="inlineStr">
@@ -49736,6 +50215,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ467" s="21" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" s="21" t="inlineStr">
@@ -49852,6 +50332,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ468" s="21" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" s="21" t="inlineStr">
@@ -49968,6 +50449,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ469" s="21" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" s="21" t="inlineStr">
@@ -50084,6 +50566,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ470" s="21" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" s="21" t="inlineStr">
@@ -50200,6 +50683,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ471" s="21" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" s="21" t="inlineStr">
@@ -50316,6 +50800,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ472" s="21" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" s="21" t="inlineStr">
@@ -50432,6 +50917,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ473" s="21" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" s="21" t="inlineStr">
@@ -50548,6 +51034,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ474" s="21" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" s="21" t="inlineStr">
@@ -50664,6 +51151,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ475" s="21" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" s="21" t="inlineStr">
@@ -50780,6 +51268,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ476" s="21" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" s="21" t="inlineStr">
@@ -50896,6 +51385,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ477" s="21" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" s="21" t="inlineStr">
@@ -51012,6 +51502,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ478" s="21" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" s="21" t="inlineStr">
@@ -51128,6 +51619,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ479" s="21" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" s="21" t="inlineStr">
@@ -51244,6 +51736,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ480" s="21" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" s="21" t="inlineStr">
@@ -51360,6 +51853,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ481" s="21" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" s="21" t="inlineStr">
@@ -51476,6 +51970,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ482" s="21" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" s="21" t="inlineStr">
@@ -51592,6 +52087,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ483" s="21" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" s="21" t="inlineStr">
@@ -51708,6 +52204,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ484" s="21" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" s="21" t="inlineStr">
@@ -51824,6 +52321,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ485" s="21" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" s="21" t="inlineStr">
@@ -51940,6 +52438,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ486" s="21" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" s="21" t="inlineStr">
@@ -52056,6 +52555,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ487" s="21" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" s="21" t="inlineStr">
@@ -52172,6 +52672,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ488" s="21" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" s="21" t="inlineStr">
@@ -52288,6 +52789,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ489" s="21" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" s="21" t="inlineStr">
@@ -52404,6 +52906,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ490" s="21" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" s="21" t="inlineStr">
@@ -52520,6 +53023,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ491" s="21" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" s="21" t="inlineStr">
@@ -52636,6 +53140,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ492" s="21" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" s="21" t="inlineStr">
@@ -52752,6 +53257,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ493" s="21" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" s="21" t="inlineStr">
@@ -52868,6 +53374,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ494" s="21" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" s="21" t="inlineStr">
@@ -52984,6 +53491,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ495" s="21" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" s="21" t="inlineStr">
@@ -53100,6 +53608,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ496" s="21" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" s="21" t="inlineStr">
@@ -53216,6 +53725,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ497" s="21" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" s="21" t="inlineStr">
@@ -53332,6 +53842,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ498" s="21" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" s="21" t="inlineStr">
@@ -53448,6 +53959,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ499" s="21" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" s="21" t="inlineStr">
@@ -53564,6 +54076,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ500" s="21" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" s="21" t="inlineStr">
@@ -53680,6 +54193,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ501" s="21" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" s="21" t="inlineStr">
@@ -53796,6 +54310,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ502" s="21" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" s="21" t="inlineStr">
@@ -53912,6 +54427,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ503" s="21" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" s="21" t="inlineStr">
@@ -54028,6 +54544,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ504" s="21" t="inlineStr"/>
     </row>
     <row r="505">
       <c r="A505" s="21" t="inlineStr">
@@ -54144,6 +54661,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ505" s="21" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" s="21" t="inlineStr">
@@ -54260,6 +54778,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ506" s="21" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" s="21" t="inlineStr">
@@ -54376,6 +54895,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ507" s="21" t="inlineStr"/>
     </row>
     <row r="508">
       <c r="A508" s="21" t="inlineStr">
@@ -54492,6 +55012,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ508" s="21" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" s="21" t="inlineStr">
@@ -54608,6 +55129,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ509" s="21" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" s="21" t="inlineStr">
@@ -54724,6 +55246,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ510" s="21" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" s="21" t="inlineStr">
@@ -54840,6 +55363,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ511" s="21" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" s="21" t="inlineStr">
@@ -54956,6 +55480,7 @@
           <t>MISSING(&gt;30d)</t>
         </is>
       </c>
+      <c r="AQ512" s="21" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" s="21" t="inlineStr">
@@ -55074,6 +55599,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ513" s="21" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" s="21" t="inlineStr">
@@ -55204,6 +55730,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ514" s="21" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" s="21" t="inlineStr">
@@ -55334,6 +55861,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ515" s="21" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" s="21" t="inlineStr">
@@ -55466,6 +55994,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ516" s="21" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" s="21" t="inlineStr">
@@ -55602,6 +56131,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ517" s="21" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" s="21" t="inlineStr">
@@ -55738,6 +56268,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ518" s="21" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" s="21" t="inlineStr">
@@ -55876,6 +56407,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ519" s="21" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" s="21" t="inlineStr">
@@ -56014,6 +56546,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ520" s="21" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" s="21" t="inlineStr">
@@ -56154,6 +56687,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ521" s="21" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" s="21" t="inlineStr">
@@ -56294,6 +56828,7 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ522" s="21" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" s="21" t="inlineStr">
@@ -56434,6 +56969,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ523" s="21" t="n">
+        <v>0.0701</v>
+      </c>
     </row>
     <row r="524">
       <c r="A524" s="21" t="inlineStr">
@@ -56574,6 +57112,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ524" s="21" t="n">
+        <v>0.1317</v>
+      </c>
     </row>
     <row r="525">
       <c r="A525" s="21" t="inlineStr">
@@ -56693,9 +57234,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL525" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL525" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM525" s="21" t="inlineStr">
@@ -56703,7 +57244,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN525" s="21" t="inlineStr"/>
+      <c r="AN525" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.463,A3-slope=1.089,A4=True,A5-oicp=?) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO525" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -56713,6 +57258,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ525" s="21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="526">
@@ -56833,9 +57381,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL526" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL526" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM526" s="21" t="inlineStr">
@@ -56843,7 +57391,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN526" s="21" t="inlineStr"/>
+      <c r="AN526" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.472,A3-slope=1.112,A4=False,A5-oicp=?) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO526" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -56853,6 +57405,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ526" s="21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="527">
@@ -56973,9 +57528,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL527" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL527" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM527" s="21" t="inlineStr">
@@ -56983,7 +57538,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN527" s="21" t="inlineStr"/>
+      <c r="AN527" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.466,A3-slope=0.935,A4=False,A5-oicp=0.176) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO527" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -56993,6 +57552,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ527" s="21" t="n">
+        <v>0.1759</v>
       </c>
     </row>
     <row r="528">
@@ -57113,9 +57675,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL528" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL528" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM528" s="21" t="inlineStr">
@@ -57123,7 +57685,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN528" s="21" t="inlineStr"/>
+      <c r="AN528" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.464,A3-slope=0.981,A4=False,A5-oicp=?) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO528" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -57133,6 +57699,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ528" s="21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="529">
@@ -57253,9 +57822,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL529" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL529" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM529" s="21" t="inlineStr">
@@ -57263,7 +57832,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN529" s="21" t="inlineStr"/>
+      <c r="AN529" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.464,A3-slope=1.003,A4=True,A5-oicp=0.536) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO529" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -57273,6 +57846,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ529" s="21" t="n">
+        <v>0.5358000000000001</v>
       </c>
     </row>
     <row r="530">
@@ -57414,6 +57990,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ530" s="21" t="n">
+        <v>0.0126</v>
+      </c>
     </row>
     <row r="531">
       <c r="A531" s="21" t="inlineStr">
@@ -57554,6 +58133,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ531" s="21" t="n">
+        <v>0.1143</v>
+      </c>
     </row>
     <row r="532">
       <c r="A532" s="21" t="inlineStr">
@@ -57694,6 +58276,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ532" s="21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="533">
       <c r="A533" s="21" t="inlineStr">
@@ -57834,6 +58419,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ533" s="21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="534">
       <c r="A534" s="21" t="inlineStr">
@@ -57974,6 +58562,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ534" s="21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="535">
       <c r="A535" s="21" t="inlineStr">
@@ -58093,9 +58684,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL535" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL535" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM535" s="21" t="inlineStr">
@@ -58103,7 +58694,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN535" s="21" t="inlineStr"/>
+      <c r="AN535" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.593,A3-slope=0.882,A4=False,A5-oicp=0.074) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO535" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -58113,6 +58708,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ535" s="21" t="n">
+        <v>0.074</v>
       </c>
     </row>
     <row r="536">
@@ -58233,9 +58831,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL536" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL536" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM536" s="21" t="inlineStr">
@@ -58243,7 +58841,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN536" s="21" t="inlineStr"/>
+      <c r="AN536" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.576,A3-slope=0.866,A4=False,A5-oicp=0.051) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO536" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -58253,6 +58855,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ536" s="21" t="n">
+        <v>0.051</v>
       </c>
     </row>
     <row r="537">
@@ -58385,7 +58990,7 @@
       </c>
       <c r="AN537" s="21" t="inlineStr">
         <is>
-          <t>A(A1=True,A2-ratio=True,A3=True,A4=True,A5=True) — gom_detect_spec v1.1 CHUA KY</t>
+          <t>A(A1=True,A2-avg5gLSR=0.568,A3-slope=0.933,A4=True,A5-oicp=0.079) — spec v1.4 ky 08/08</t>
         </is>
       </c>
       <c r="AO537" s="21" t="inlineStr">
@@ -58397,6 +59002,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ537" s="21" t="n">
+        <v>0.0788</v>
       </c>
     </row>
     <row r="538">
@@ -58538,6 +59146,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ538" s="21" t="n">
+        <v>0.6966</v>
+      </c>
     </row>
     <row r="539">
       <c r="A539" s="21" t="inlineStr">
@@ -58657,9 +59268,9 @@
           <t>ABSTAIN(Nansen_LOCKED)</t>
         </is>
       </c>
-      <c r="AL539" s="21" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="AL539" s="22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AM539" s="21" t="inlineStr">
@@ -58667,7 +59278,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AN539" s="21" t="inlineStr"/>
+      <c r="AN539" s="21" t="inlineStr">
+        <is>
+          <t>A(A1=True,A2-avg5gLSR=0.644,A3-slope=1.091,A4=True,A5-oicp=0.41) — spec v1.4 ky 08/08</t>
+        </is>
+      </c>
       <c r="AO539" s="21" t="inlineStr">
         <is>
           <t>fapi_klines_1d</t>
@@ -58677,6 +59292,9 @@
         <is>
           <t>fapi_LSR_30d</t>
         </is>
+      </c>
+      <c r="AQ539" s="21" t="n">
+        <v>0.41</v>
       </c>
     </row>
     <row r="540">
@@ -58818,6 +59436,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ540" s="21" t="n">
+        <v>0.5454</v>
+      </c>
     </row>
     <row r="541">
       <c r="A541" s="21" t="inlineStr">
@@ -58958,6 +59579,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ541" s="21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="542">
       <c r="A542" s="21" t="inlineStr">
@@ -59098,6 +59722,9 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ542" s="21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="543">
       <c r="A543" s="21" t="inlineStr">
@@ -59106,25 +59733,25 @@
         </is>
       </c>
       <c r="B543" s="21" t="n">
-        <v>0.19530333</v>
+        <v>0.20423667</v>
       </c>
       <c r="C543" s="21" t="n">
         <v>0.19656</v>
       </c>
       <c r="D543" s="21" t="n">
-        <v>0.21362</v>
+        <v>0.22785</v>
       </c>
       <c r="E543" s="21" t="n">
         <v>0.1656</v>
       </c>
       <c r="F543" s="21" t="n">
-        <v>0.20669</v>
+        <v>0.21926</v>
       </c>
       <c r="G543" s="21" t="n">
-        <v>128294844.628611</v>
+        <v>137936646.297419</v>
       </c>
       <c r="H543" s="21" t="n">
-        <v>50.2</v>
+        <v>50.47</v>
       </c>
       <c r="I543" s="21" t="n">
         <v>8.379999999999999e-06</v>
@@ -59150,7 +59777,9 @@
       <c r="P543" s="21" t="b">
         <v>1</v>
       </c>
-      <c r="Q543" s="21" t="inlineStr"/>
+      <c r="Q543" s="21" t="n">
+        <v>11.5486</v>
+      </c>
       <c r="R543" s="21" t="n">
         <v>0</v>
       </c>
@@ -59161,7 +59790,7 @@
         <v>3.589</v>
       </c>
       <c r="U543" s="21" t="n">
-        <v>28.27</v>
+        <v>30.4</v>
       </c>
       <c r="V543" s="21" t="n">
         <v>1.3154</v>
@@ -59189,13 +59818,13 @@
       </c>
       <c r="AD543" s="21" t="inlineStr"/>
       <c r="AE543" s="21" t="n">
-        <v>11663623.52438</v>
+        <v>12819953.23067</v>
       </c>
       <c r="AF543" s="21" t="n">
-        <v>46.96</v>
+        <v>47.91</v>
       </c>
       <c r="AG543" s="21" t="n">
-        <v>0.091</v>
+        <v>0.093</v>
       </c>
       <c r="AH543" s="21" t="inlineStr">
         <is>
@@ -59238,9 +59867,13 @@
           <t>fapi_LSR_30d</t>
         </is>
       </c>
+      <c r="AQ543" s="21" t="n">
+        <v>0.5255</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="AQ1"/>
     <mergeCell ref="AL1:AN1"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="AI1:AJ1"/>
@@ -59260,7 +59893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="12" min="1" max="1"/>
@@ -59573,6 +60206,9 @@
           <t>fapi klines+LSR csv</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>